<commit_message>
Bake SharePoint Excel values to fix #WERT!
Excel Online cannot resolve cross-workbook links. Replace formula cells
in the hub and dateien/*.xlsx with cached numbers from the Import workbook,
refresh download/NEUSTART ZIPs, and document re-upload steps.

Co-authored-by: fabsieb-boop <fabsieb-boop@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/workbook-split/dateien/Abgrenzungen.xlsx
+++ b/docs/workbook-split/dateien/Abgrenzungen.xlsx
@@ -686,9 +686,8 @@
       <c r="F7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="6">
-        <f>SUM(E7:F7)</f>
-        <v/>
+      <c r="G7" s="6" t="n">
+        <v>-280</v>
       </c>
       <c r="H7" s="1" t="n"/>
       <c r="I7" s="1" t="n"/>
@@ -717,9 +716,8 @@
       <c r="F8" s="6" t="n">
         <v>-8.1</v>
       </c>
-      <c r="G8" s="6">
-        <f>SUM(E8:F8)</f>
-        <v/>
+      <c r="G8" s="6" t="n">
+        <v>-956.1</v>
       </c>
       <c r="H8" s="1" t="n"/>
       <c r="I8" s="1" t="n"/>
@@ -748,9 +746,8 @@
       <c r="F9" s="6" t="n">
         <v>8545.030000000001</v>
       </c>
-      <c r="G9" s="6">
-        <f>SUM(E9:F9)</f>
-        <v/>
+      <c r="G9" s="6" t="n">
+        <v>-21765.48</v>
       </c>
       <c r="H9" s="1" t="n"/>
       <c r="I9" s="1" t="n"/>
@@ -779,9 +776,8 @@
       <c r="F10" s="6" t="n">
         <v>-12968</v>
       </c>
-      <c r="G10" s="6">
-        <f>SUM(E10:F10)</f>
-        <v/>
+      <c r="G10" s="6" t="n">
+        <v>-14873</v>
       </c>
       <c r="H10" s="1" t="n"/>
       <c r="I10" s="1" t="n"/>
@@ -810,9 +806,8 @@
       <c r="F11" s="6" t="n">
         <v>-64651.92</v>
       </c>
-      <c r="G11" s="6">
-        <f>SUM(E11:F11)</f>
-        <v/>
+      <c r="G11" s="6" t="n">
+        <v>-73755.92</v>
       </c>
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="1" t="n"/>
@@ -841,9 +836,8 @@
       <c r="F12" s="6" t="n">
         <v>12968</v>
       </c>
-      <c r="G12" s="6">
-        <f>SUM(E12:F12)</f>
-        <v/>
+      <c r="G12" s="6" t="n">
+        <v>14873</v>
       </c>
       <c r="H12" s="1" t="n"/>
       <c r="I12" s="1" t="n"/>
@@ -872,9 +866,8 @@
       <c r="F13" s="6" t="n">
         <v>64651.92</v>
       </c>
-      <c r="G13" s="6">
-        <f>SUM(E13:F13)</f>
-        <v/>
+      <c r="G13" s="6" t="n">
+        <v>73755.92</v>
       </c>
       <c r="H13" s="1" t="n"/>
       <c r="I13" s="1" t="n"/>
@@ -903,9 +896,8 @@
       <c r="F14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="6">
-        <f>SUM(E14:F14)</f>
-        <v/>
+      <c r="G14" s="6" t="n">
+        <v>763.4299999999999</v>
       </c>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="1" t="n"/>
@@ -934,9 +926,8 @@
       <c r="F15" s="6" t="n">
         <v>-42350</v>
       </c>
-      <c r="G15" s="6">
-        <f>SUM(E15:F15)</f>
-        <v/>
+      <c r="G15" s="6" t="n">
+        <v>-42350</v>
       </c>
       <c r="H15" s="1" t="n"/>
       <c r="I15" s="1" t="n"/>
@@ -965,9 +956,8 @@
       <c r="F16" s="6" t="n">
         <v>-185038</v>
       </c>
-      <c r="G16" s="6">
-        <f>SUM(E16:F16)</f>
-        <v/>
+      <c r="G16" s="6" t="n">
+        <v>-185038</v>
       </c>
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="1" t="n"/>
@@ -996,9 +986,8 @@
       <c r="F17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="6">
-        <f>SUM(E17:F17)</f>
-        <v/>
+      <c r="G17" s="6" t="n">
+        <v>-3874379.85</v>
       </c>
       <c r="H17" s="1" t="n"/>
       <c r="I17" s="1" t="n"/>
@@ -1027,9 +1016,8 @@
       <c r="F18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="6">
-        <f>SUM(E18:F18)</f>
-        <v/>
+      <c r="G18" s="6" t="n">
+        <v>2702877.8</v>
       </c>
       <c r="H18" s="1" t="n"/>
       <c r="I18" s="1" t="n"/>
@@ -1058,9 +1046,8 @@
       <c r="F19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="6">
-        <f>SUM(E19:F19)</f>
-        <v/>
+      <c r="G19" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H19" s="1" t="n"/>
       <c r="I19" s="1" t="n"/>
@@ -1089,9 +1076,8 @@
       <c r="F20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="6">
-        <f>SUM(E20:F20)</f>
-        <v/>
+      <c r="G20" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H20" s="1" t="n"/>
       <c r="I20" s="1" t="n"/>
@@ -1120,9 +1106,8 @@
       <c r="F21" s="6" t="n">
         <v>-1181.41</v>
       </c>
-      <c r="G21" s="6">
-        <f>SUM(E21:F21)</f>
-        <v/>
+      <c r="G21" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H21" s="1" t="n"/>
       <c r="I21" s="1" t="n"/>
@@ -1151,9 +1136,8 @@
       <c r="F22" s="6" t="n">
         <v>343774.94</v>
       </c>
-      <c r="G22" s="6">
-        <f>SUM(E22:F22)</f>
-        <v/>
+      <c r="G22" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H22" s="1" t="n"/>
       <c r="I22" s="1" t="n"/>
@@ -1182,9 +1166,8 @@
       <c r="F23" s="6" t="n">
         <v>59943.4</v>
       </c>
-      <c r="G23" s="6">
-        <f>SUM(E23:F23)</f>
-        <v/>
+      <c r="G23" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H23" s="1" t="n"/>
       <c r="I23" s="1" t="n"/>
@@ -1213,9 +1196,8 @@
       <c r="F24" s="6" t="n">
         <v>1181.41</v>
       </c>
-      <c r="G24" s="6">
-        <f>SUM(E24:F24)</f>
-        <v/>
+      <c r="G24" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H24" s="1" t="n"/>
       <c r="I24" s="1" t="n"/>
@@ -1244,9 +1226,8 @@
       <c r="F25" s="6" t="n">
         <v>-343774.94</v>
       </c>
-      <c r="G25" s="6">
-        <f>SUM(E25:F25)</f>
-        <v/>
+      <c r="G25" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H25" s="1" t="n"/>
       <c r="I25" s="1" t="n"/>
@@ -1275,9 +1256,8 @@
       <c r="F26" s="6" t="n">
         <v>992.0599999999999</v>
       </c>
-      <c r="G26" s="6">
-        <f>SUM(E26:F26)</f>
-        <v/>
+      <c r="G26" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H26" s="1" t="n"/>
       <c r="I26" s="1" t="n"/>
@@ -1306,9 +1286,8 @@
       <c r="F27" s="6" t="n">
         <v>1645.8</v>
       </c>
-      <c r="G27" s="6">
-        <f>SUM(E27:F27)</f>
-        <v/>
+      <c r="G27" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H27" s="1" t="n"/>
       <c r="I27" s="1" t="n"/>
@@ -1337,9 +1316,8 @@
       <c r="F28" s="6" t="n">
         <v>88700</v>
       </c>
-      <c r="G28" s="6">
-        <f>SUM(E28:F28)</f>
-        <v/>
+      <c r="G28" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H28" s="1" t="n"/>
       <c r="I28" s="1" t="n"/>
@@ -1368,9 +1346,8 @@
       <c r="F29" s="6" t="n">
         <v>22148</v>
       </c>
-      <c r="G29" s="6">
-        <f>SUM(E29:F29)</f>
-        <v/>
+      <c r="G29" s="6" t="n">
+        <v>-11182</v>
       </c>
       <c r="H29" s="1" t="n"/>
       <c r="I29" s="1" t="n"/>
@@ -1399,9 +1376,8 @@
       <c r="F30" s="6" t="n">
         <v>700</v>
       </c>
-      <c r="G30" s="6">
-        <f>SUM(E30:F30)</f>
-        <v/>
+      <c r="G30" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H30" s="1" t="n"/>
       <c r="I30" s="1" t="n"/>
@@ -1430,9 +1406,8 @@
       <c r="F31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="6">
-        <f>SUM(E31:F31)</f>
-        <v/>
+      <c r="G31" s="6" t="n">
+        <v>7519</v>
       </c>
       <c r="H31" s="1" t="n"/>
       <c r="I31" s="1" t="n"/>
@@ -2572,6 +2547,8 @@
       </c>
     </row>
     <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
     <row r="124">
       <c r="C124" t="inlineStr">
         <is>

</xml_diff>